<commit_message>
Planilha 17: variação de horas e caixa só quando o mês fechou (Config), telas regeneradas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/17-painel-do-escritorio.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/17-painel-do-escritorio.xlsx
@@ -1519,7 +1519,7 @@
         <v>—</v>
       </c>
       <c r="G15" s="22" t="str">
-        <f>IF(OR(C15="—",F15="—",F15=0),"—",(C15-F15)/ABS(F15))</f>
+        <f>(IF(OR(C15="—",F15="—",F15=0),"—",(C15-F15)/ABS(F15)))</f>
         <v>—</v>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
         <v>—</v>
       </c>
       <c r="G16" s="22" t="str">
-        <f>IF(OR(C16="—",F16="—",F16=0),"—",(C16-F16)/ABS(F16))</f>
+        <f>(IF(OR(C16="—",F16="—",F16=0),"—",(C16-F16)/ABS(F16)))</f>
         <v>—</v>
       </c>
     </row>
@@ -1572,9 +1572,9 @@
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$D$5:$D$16,Config!$B$8-1)="","—",INDEX(Histórico!$D$5:$D$16,Config!$B$8-1)))</f>
         <v>304</v>
       </c>
-      <c r="G17" s="22">
-        <f>IF(OR(C17="—",F17="—",F17=0),"—",(C17-F17)/ABS(F17))</f>
-        <v>-0.639802631578947</v>
+      <c r="G17" s="22" t="str">
+        <f>IF(Config!$B$10&lt;&gt;"Sim","no fechamento",IF(OR(C17="—",F17="—",F17=0),"—",(C17-F17)/ABS(F17)))</f>
+        <v>no fechamento</v>
       </c>
     </row>
     <row r="18">
@@ -1599,9 +1599,9 @@
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$E$5:$E$16,Config!$B$8-1)="","—",INDEX(Histórico!$E$5:$E$16,Config!$B$8-1)))</f>
         <v>248</v>
       </c>
-      <c r="G18" s="22">
-        <f>IF(OR(C18="—",F18="—",F18=0),"—",(C18-F18)/ABS(F18))</f>
-        <v>-0.649193548387097</v>
+      <c r="G18" s="22" t="str">
+        <f>IF(Config!$B$10&lt;&gt;"Sim","no fechamento",IF(OR(C18="—",F18="—",F18=0),"—",(C18-F18)/ABS(F18)))</f>
+        <v>no fechamento</v>
       </c>
     </row>
     <row r="19">
@@ -1627,7 +1627,7 @@
         <v>0.815789473684211</v>
       </c>
       <c r="G19" s="25">
-        <f>IF(OR(C19="—",F19="—"),"—",(C19-F19)*100)</f>
+        <f>(IF(OR(C19="—",F19="—"),"—",(C19-F19)*100))</f>
         <v>-2.12689257390051</v>
       </c>
     </row>
@@ -1653,9 +1653,9 @@
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$G$5:$G$16,Config!$B$8-1)="","—",INDEX(Histórico!$G$5:$G$16,Config!$B$8-1)))</f>
         <v>26900</v>
       </c>
-      <c r="G20" s="22">
-        <f>IF(OR(C20="—",F20="—",F20=0),"—",(C20-F20)/ABS(F20))</f>
-        <v>-0.805947955390335</v>
+      <c r="G20" s="22" t="str">
+        <f>IF(Config!$B$10&lt;&gt;"Sim","no fechamento",IF(OR(C20="—",F20="—",F20=0),"—",(C20-F20)/ABS(F20)))</f>
+        <v>no fechamento</v>
       </c>
     </row>
     <row r="21">
@@ -1680,9 +1680,9 @@
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$H$5:$H$16,Config!$B$8-1)="","—",INDEX(Histórico!$H$5:$H$16,Config!$B$8-1)))</f>
         <v>21897</v>
       </c>
-      <c r="G21" s="22">
-        <f>IF(OR(C21="—",F21="—",F21=0),"—",(C21-F21)/ABS(F21))</f>
-        <v>-0.75704434397406</v>
+      <c r="G21" s="22" t="str">
+        <f>IF(Config!$B$10&lt;&gt;"Sim","no fechamento",IF(OR(C21="—",F21="—",F21=0),"—",(C21-F21)/ABS(F21)))</f>
+        <v>no fechamento</v>
       </c>
     </row>
     <row r="22">
@@ -1707,9 +1707,9 @@
         <f>IF(Config!$B$8&lt;=1,"—",IF(INDEX(Histórico!$I$5:$I$16,Config!$B$8-1)="","—",INDEX(Histórico!$I$5:$I$16,Config!$B$8-1)))</f>
         <v>5003</v>
       </c>
-      <c r="G22" s="22">
-        <f>IF(OR(C22="—",F22="—",F22=0),"—",(C22-F22)/ABS(F22))</f>
-        <v>-1.01998800719568</v>
+      <c r="G22" s="22" t="str">
+        <f>IF(Config!$B$10&lt;&gt;"Sim","no fechamento",IF(OR(C22="—",F22="—",F22=0),"—",(C22-F22)/ABS(F22)))</f>
+        <v>no fechamento</v>
       </c>
     </row>
     <row r="23">
@@ -1735,7 +1735,7 @@
         <v>117210</v>
       </c>
       <c r="G23" s="22">
-        <f>IF(OR(C23="—",F23="—",F23=0),"—",(C23-F23)/ABS(F23))</f>
+        <f>(IF(OR(C23="—",F23="—",F23=0),"—",(C23-F23)/ABS(F23)))</f>
         <v>-0.0445354491937548</v>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
         <v>12500</v>
       </c>
       <c r="G24" s="22">
-        <f>IF(OR(C24="—",F24="—",F24=0),"—",(C24-F24)/ABS(F24))</f>
+        <f>(IF(OR(C24="—",F24="—",F24=0),"—",(C24-F24)/ABS(F24)))</f>
         <v>0.1584</v>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
         <v>0.0447723772341416</v>
       </c>
       <c r="G25" s="25">
-        <f>IF(OR(C25="—",F25="—"),"—",(C25-F25)*100)</f>
+        <f>(IF(OR(C25="—",F25="—"),"—",(C25-F25)*100))</f>
         <v>0.578804736168925</v>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
         <v>5</v>
       </c>
       <c r="G26" s="22">
-        <f>IF(OR(C26="—",F26="—",F26=0),"—",(C26-F26)/ABS(F26))</f>
+        <f>(IF(OR(C26="—",F26="—",F26=0),"—",(C26-F26)/ABS(F26)))</f>
         <v>0.8</v>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
         <v>46900</v>
       </c>
       <c r="G27" s="22">
-        <f>IF(OR(C27="—",F27="—",F27=0),"—",(C27-F27)/ABS(F27))</f>
+        <f>(IF(OR(C27="—",F27="—",F27=0),"—",(C27-F27)/ABS(F27)))</f>
         <v>0.554371002132196</v>
       </c>
     </row>
@@ -1870,14 +1870,14 @@
         <v>30</v>
       </c>
       <c r="G28" s="22">
-        <f>IF(OR(C28="—",F28="—",F28=0),"—",(C28-F28)/ABS(F28))</f>
+        <f>(IF(OR(C28="—",F28="—",F28=0),"—",(C28-F28)/ABS(F28)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>Fora do alvo primeiro: prazos atrasados e vencido pedem ação na segunda-feira (planilhas 01 e 14). Variação de indicadores em % é em pontos percentuais (p.p.). No meio do mês, horas e caixa ainda estão parciais: compare com o mês anterior só no fechamento. A planilha avisa; o controle é do escritório.</t>
+          <t>Fora do alvo primeiro: prazos atrasados e vencido pedem ação na segunda-feira (planilhas 01 e 14). Variação de indicadores em % é em pontos percentuais (p.p.). No meio do mês, horas e caixa ainda estão parciais: a variação deles só aparece quando Config diz que o mês fechou. A planilha avisa; o controle é do escritório.</t>
         </is>
       </c>
     </row>
@@ -2237,6 +2237,16 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Mês do painel já fechou? (Sim/Não)</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
           <t>Junho</t>
@@ -2246,7 +2256,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Use a mesma planilha o ano inteiro: troque o mês aqui e, no fim de cada mês, copie a linha de Dados para o Histórico.</t>
+          <t>Use a mesma planilha o ano inteiro: troque o mês aqui e, no fim de cada mês, copie a linha de Dados para o Histórico. Enquanto o mês não fecha, horas e caixa são parciais e o Painel não os compara com o mês anterior (marque Sim no fechamento).</t>
         </is>
       </c>
       <c r="D11" s="32" t="inlineStr">
@@ -2296,7 +2306,10 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>=Config!$D$5:$D$16</formula1>
     </dataValidation>

</xml_diff>